<commit_message>
ajout image, buget et planning
</commit_message>
<xml_diff>
--- a/docs/rapport/assets/Planning.xlsx
+++ b/docs/rapport/assets/Planning.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30006"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30128"/>
   <workbookPr showInkAnnotation="0" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://hessoit-my.sharepoint.com/personal/tom_berthoud_hes-so_ch/Documents/ProjetMultiScaner3D/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="343" documentId="8_{4C4FB89F-EA90-4D91-AE4E-64D724AF4ABA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{14A7C3C5-AC77-4A9A-96D8-C25E6A95C036}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{B2DD41F8-4A25-4EF1-A27E-060334FF0A1E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="13872" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Tâches" sheetId="4" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Tâches!$A$1:$Z$67</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Tâches!$A$1:$Z$69</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -65,7 +65,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="138">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="144">
   <si>
     <t>N°</t>
   </si>
@@ -340,6 +340,12 @@
     <t>Alimentation 230V → régulation + sécurité</t>
   </si>
   <si>
+    <t>T20.20.45</t>
+  </si>
+  <si>
+    <t>Câblage au propre</t>
+  </si>
+  <si>
     <t>T20.20.50</t>
   </si>
   <si>
@@ -403,10 +409,22 @@
     <t>Interface utilisateur (native et/ou web)</t>
   </si>
   <si>
+    <t>T30.15</t>
+  </si>
+  <si>
+    <t>Amélioration qualité du scan (calibration, bruit, résolution)</t>
+  </si>
+  <si>
+    <t>Tom / Tous</t>
+  </si>
+  <si>
     <t>T30.20</t>
   </si>
   <si>
     <t>Intégration complète (UI ↔ algo ↔ hardware)</t>
+  </si>
+  <si>
+    <t>Jason Hadrien Tom</t>
   </si>
   <si>
     <t>T30.30</t>
@@ -1044,7 +1062,7 @@
     <we:reference id="WA200009404" version="1.0.0.5" store="WA200009404" storeType="OMEX"/>
   </we:alternateReferences>
   <we:properties>
-    <we:property name="Office.AutoShowTaskpaneWithDocument" value="true"/>
+    <we:property name="claude.fileId" value="&quot;78cb3119-6ee7-4619-9b55-ce44c81d7b46&quot;"/>
   </we:properties>
   <we:bindings/>
   <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
@@ -1061,12 +1079,12 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:Z61"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="12.4"/>
+  <dimension ref="A1:Z63"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="12.75" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="13.140625" style="24" customWidth="1"/>
     <col min="2" max="2" width="4.140625" style="5" customWidth="1"/>
-    <col min="3" max="3" width="4.140625" style="25" customWidth="1"/>
+    <col min="3" max="3" width="49.7109375" style="25" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="19.85546875" style="25" customWidth="1"/>
     <col min="5" max="5" width="44.28515625" style="25" customWidth="1"/>
     <col min="6" max="6" width="23.5703125" style="25" customWidth="1"/>
@@ -1077,7 +1095,7 @@
     <col min="26" max="26" width="11.42578125" style="30" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:26" s="5" customFormat="1" ht="12.6" thickBot="1">
+    <row r="1" spans="1:26" s="5" customFormat="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1184,7 +1202,7 @@
       <c r="X2" s="11"/>
       <c r="Y2" s="9"/>
       <c r="Z2" s="28">
-        <f t="shared" ref="Z2:Z59" si="0">G2-X2-Y2</f>
+        <f>G2-X2-Y2</f>
         <v>0</v>
       </c>
     </row>
@@ -1222,11 +1240,11 @@
       </c>
       <c r="Y3" s="9"/>
       <c r="Z3" s="28">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:26" ht="61.5">
+        <f>G3-X3-Y3</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:26" ht="60">
       <c r="A4" s="6" t="s">
         <v>28</v>
       </c>
@@ -1263,12 +1281,12 @@
       <c r="V4" s="10"/>
       <c r="W4" s="10"/>
       <c r="X4" s="11">
-        <f t="shared" ref="X4:X18" si="1">SUM(H4:W4)</f>
+        <f t="shared" ref="X4:X18" si="0">SUM(H4:W4)</f>
         <v>3</v>
       </c>
       <c r="Y4" s="9"/>
       <c r="Z4" s="28">
-        <f t="shared" ref="Z4:Z30" si="2">G4-X4-Y4</f>
+        <f>G4-X4-Y4</f>
         <v>0</v>
       </c>
     </row>
@@ -1309,12 +1327,12 @@
       <c r="V5" s="10"/>
       <c r="W5" s="10"/>
       <c r="X5" s="11">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>5</v>
       </c>
       <c r="Y5" s="9"/>
       <c r="Z5" s="28">
-        <f t="shared" si="2"/>
+        <f>G5-X5-Y5</f>
         <v>0</v>
       </c>
     </row>
@@ -1347,12 +1365,12 @@
       <c r="V6" s="10"/>
       <c r="W6" s="10"/>
       <c r="X6" s="11">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="Y6" s="9"/>
       <c r="Z6" s="28">
-        <f t="shared" si="2"/>
+        <f>G6-X6-Y6</f>
         <v>0</v>
       </c>
     </row>
@@ -1389,12 +1407,14 @@
       <c r="V7" s="10"/>
       <c r="W7" s="10"/>
       <c r="X7" s="11">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="Y7" s="9"/>
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="Y7" s="9">
+        <v>0</v>
+      </c>
       <c r="Z7" s="28">
-        <f t="shared" si="2"/>
+        <f>G7-X7-Y7</f>
         <v>3</v>
       </c>
     </row>
@@ -1431,12 +1451,12 @@
       <c r="V8" s="10"/>
       <c r="W8" s="10"/>
       <c r="X8" s="11">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>3</v>
       </c>
       <c r="Y8" s="9"/>
       <c r="Z8" s="28">
-        <f t="shared" si="2"/>
+        <f>G8-X8-Y8</f>
         <v>0</v>
       </c>
     </row>
@@ -1473,12 +1493,12 @@
       <c r="V9" s="10"/>
       <c r="W9" s="10"/>
       <c r="X9" s="11">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>4</v>
       </c>
       <c r="Y9" s="9"/>
       <c r="Z9" s="28">
-        <f t="shared" si="2"/>
+        <f>G9-X9-Y9</f>
         <v>-1</v>
       </c>
     </row>
@@ -1515,12 +1535,12 @@
       <c r="V10" s="10"/>
       <c r="W10" s="10"/>
       <c r="X10" s="11">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>5</v>
       </c>
       <c r="Y10" s="9"/>
       <c r="Z10" s="28">
-        <f t="shared" si="2"/>
+        <f>G10-X10-Y10</f>
         <v>-2</v>
       </c>
     </row>
@@ -1557,16 +1577,16 @@
       <c r="V11" s="10"/>
       <c r="W11" s="10"/>
       <c r="X11" s="11">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>2</v>
       </c>
       <c r="Y11" s="9"/>
       <c r="Z11" s="28">
-        <f t="shared" si="2"/>
+        <f>G11-X11-Y11</f>
         <v>2</v>
       </c>
     </row>
-    <row r="12" spans="1:26" ht="24.6">
+    <row r="12" spans="1:26" ht="24">
       <c r="A12" s="6"/>
       <c r="B12" s="7"/>
       <c r="C12" s="8"/>
@@ -1599,9 +1619,11 @@
       <c r="V12" s="10"/>
       <c r="W12" s="10"/>
       <c r="X12" s="11"/>
-      <c r="Y12" s="9"/>
+      <c r="Y12" s="9">
+        <v>0</v>
+      </c>
       <c r="Z12" s="28">
-        <f t="shared" si="2"/>
+        <f>G12-X12-Y12</f>
         <v>3</v>
       </c>
     </row>
@@ -1640,12 +1662,12 @@
       <c r="V13" s="10"/>
       <c r="W13" s="10"/>
       <c r="X13" s="11">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>4</v>
       </c>
       <c r="Y13" s="9"/>
       <c r="Z13" s="28">
-        <f t="shared" si="2"/>
+        <f>G13-X13-Y13</f>
         <v>0</v>
       </c>
     </row>
@@ -1684,12 +1706,12 @@
       <c r="V14" s="10"/>
       <c r="W14" s="10"/>
       <c r="X14" s="11">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>4</v>
       </c>
       <c r="Y14" s="9"/>
       <c r="Z14" s="28">
-        <f t="shared" si="2"/>
+        <f>G14-X14-Y14</f>
         <v>-1</v>
       </c>
     </row>
@@ -1720,12 +1742,12 @@
       <c r="V15" s="10"/>
       <c r="W15" s="10"/>
       <c r="X15" s="11">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="Y15" s="9"/>
       <c r="Z15" s="28">
-        <f t="shared" si="2"/>
+        <f>G15-X15-Y15</f>
         <v>0</v>
       </c>
     </row>
@@ -1758,12 +1780,12 @@
       <c r="V16" s="10"/>
       <c r="W16" s="10"/>
       <c r="X16" s="11">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="Y16" s="9"/>
       <c r="Z16" s="28">
-        <f t="shared" si="2"/>
+        <f>G16-X16-Y16</f>
         <v>0</v>
       </c>
     </row>
@@ -1802,12 +1824,12 @@
       <c r="V17" s="10"/>
       <c r="W17" s="10"/>
       <c r="X17" s="11">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>2</v>
       </c>
       <c r="Y17" s="9"/>
       <c r="Z17" s="28">
-        <f t="shared" si="2"/>
+        <f>G17-X17-Y17</f>
         <v>2</v>
       </c>
     </row>
@@ -1848,12 +1870,12 @@
       <c r="V18" s="10"/>
       <c r="W18" s="10"/>
       <c r="X18" s="11">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>10</v>
       </c>
       <c r="Y18" s="9"/>
       <c r="Z18" s="28">
-        <f t="shared" si="2"/>
+        <f>G18-X18-Y18</f>
         <v>-2</v>
       </c>
     </row>
@@ -1896,12 +1918,12 @@
       <c r="V19" s="10"/>
       <c r="W19" s="10"/>
       <c r="X19" s="11">
-        <f t="shared" ref="X19:X25" si="3">SUM(H19:W19)</f>
+        <f t="shared" ref="X19:X41" si="1">SUM(H19:W19)</f>
         <v>11</v>
       </c>
       <c r="Y19" s="9"/>
       <c r="Z19" s="28">
-        <f t="shared" si="2"/>
+        <f>G19-X19-Y19</f>
         <v>-1</v>
       </c>
     </row>
@@ -1934,12 +1956,12 @@
       <c r="V20" s="10"/>
       <c r="W20" s="10"/>
       <c r="X20" s="11">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="Y20" s="9"/>
       <c r="Z20" s="28">
-        <f t="shared" si="2"/>
+        <f>G20-X20-Y20</f>
         <v>0</v>
       </c>
     </row>
@@ -1978,12 +2000,12 @@
       <c r="V21" s="10"/>
       <c r="W21" s="10"/>
       <c r="X21" s="11">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="Y21" s="9"/>
       <c r="Z21" s="28">
-        <f t="shared" si="2"/>
+        <f>G21-X21-Y21</f>
         <v>0</v>
       </c>
     </row>
@@ -2020,12 +2042,12 @@
       <c r="V22" s="10"/>
       <c r="W22" s="10"/>
       <c r="X22" s="11">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="Y22" s="9"/>
       <c r="Z22" s="28">
-        <f t="shared" si="2"/>
+        <f>G22-X22-Y22</f>
         <v>6</v>
       </c>
     </row>
@@ -2062,12 +2084,12 @@
       <c r="V23" s="10"/>
       <c r="W23" s="10"/>
       <c r="X23" s="11">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="Y23" s="9"/>
       <c r="Z23" s="28">
-        <f t="shared" si="2"/>
+        <f>G23-X23-Y23</f>
         <v>1</v>
       </c>
     </row>
@@ -2100,12 +2122,12 @@
       <c r="V24" s="10"/>
       <c r="W24" s="10"/>
       <c r="X24" s="11">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="Y24" s="9"/>
       <c r="Z24" s="28">
-        <f t="shared" si="2"/>
+        <f>G24-X24-Y24</f>
         <v>0</v>
       </c>
     </row>
@@ -2140,12 +2162,12 @@
       <c r="V25" s="10"/>
       <c r="W25" s="10"/>
       <c r="X25" s="11">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="Y25" s="9"/>
       <c r="Z25" s="28">
-        <f t="shared" si="2"/>
+        <f>G25-X25-Y25</f>
         <v>0</v>
       </c>
     </row>
@@ -2190,12 +2212,12 @@
       <c r="V26" s="10"/>
       <c r="W26" s="10"/>
       <c r="X26" s="11">
-        <f t="shared" ref="X26:X60" si="4">SUM(H26:W26)</f>
+        <f t="shared" si="1"/>
         <v>12</v>
       </c>
       <c r="Y26" s="9"/>
       <c r="Z26" s="28">
-        <f t="shared" si="2"/>
+        <f>G26-X26-Y26</f>
         <v>0</v>
       </c>
     </row>
@@ -2236,12 +2258,12 @@
       <c r="V27" s="10"/>
       <c r="W27" s="10"/>
       <c r="X27" s="11">
-        <f t="shared" si="4"/>
+        <f t="shared" si="1"/>
         <v>8</v>
       </c>
       <c r="Y27" s="9"/>
       <c r="Z27" s="28">
-        <f t="shared" si="2"/>
+        <f>G27-X27-Y27</f>
         <v>0</v>
       </c>
     </row>
@@ -2278,16 +2300,25 @@
       <c r="P28" s="10"/>
       <c r="Q28" s="10"/>
       <c r="R28" s="10"/>
-      <c r="S28" s="10"/>
-      <c r="T28" s="10"/>
+      <c r="S28" s="10">
+        <v>2</v>
+      </c>
+      <c r="T28" s="10">
+        <v>3</v>
+      </c>
       <c r="U28" s="10"/>
       <c r="V28" s="10"/>
       <c r="W28" s="10"/>
-      <c r="X28" s="11"/>
-      <c r="Y28" s="9"/>
+      <c r="X28" s="11">
+        <f t="shared" si="1"/>
+        <v>11</v>
+      </c>
+      <c r="Y28" s="9">
+        <v>0</v>
+      </c>
       <c r="Z28" s="28">
-        <f t="shared" si="2"/>
-        <v>10</v>
+        <f>G28-X28-Y28</f>
+        <v>-1</v>
       </c>
     </row>
     <row r="29" spans="1:26">
@@ -2328,11 +2359,16 @@
       <c r="U29" s="10"/>
       <c r="V29" s="10"/>
       <c r="W29" s="10"/>
-      <c r="X29" s="11"/>
-      <c r="Y29" s="9"/>
+      <c r="X29" s="11">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="Y29" s="9">
+        <v>0</v>
+      </c>
       <c r="Z29" s="28">
-        <f t="shared" si="2"/>
-        <v>5</v>
+        <f>G29-X29-Y29</f>
+        <v>0</v>
       </c>
     </row>
     <row r="30" spans="1:26">
@@ -2363,10 +2399,13 @@
       <c r="U30" s="10"/>
       <c r="V30" s="10"/>
       <c r="W30" s="10"/>
-      <c r="X30" s="11"/>
+      <c r="X30" s="11">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
       <c r="Y30" s="9"/>
       <c r="Z30" s="28">
-        <f t="shared" si="2"/>
+        <f>G30-X30-Y30</f>
         <v>0</v>
       </c>
     </row>
@@ -2394,20 +2433,25 @@
       <c r="M31" s="10">
         <v>3</v>
       </c>
-      <c r="N31" s="10">
-        <v>3</v>
-      </c>
+      <c r="N31" s="10"/>
       <c r="O31" s="10"/>
       <c r="P31" s="10"/>
       <c r="Q31" s="10"/>
-      <c r="R31" s="10"/>
+      <c r="R31" s="10">
+        <v>3</v>
+      </c>
       <c r="S31" s="10"/>
       <c r="T31" s="10"/>
       <c r="U31" s="10"/>
       <c r="V31" s="10"/>
       <c r="W31" s="10"/>
-      <c r="X31" s="11"/>
-      <c r="Y31" s="9"/>
+      <c r="X31" s="11">
+        <f t="shared" si="1"/>
+        <v>6</v>
+      </c>
+      <c r="Y31" s="9">
+        <v>0</v>
+      </c>
       <c r="Z31" s="28"/>
     </row>
     <row r="32" spans="1:26">
@@ -2444,8 +2488,13 @@
       <c r="U32" s="10"/>
       <c r="V32" s="10"/>
       <c r="W32" s="10"/>
-      <c r="X32" s="11"/>
-      <c r="Y32" s="9"/>
+      <c r="X32" s="11">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="Y32" s="9">
+        <v>0</v>
+      </c>
       <c r="Z32" s="28"/>
     </row>
     <row r="33" spans="1:26">
@@ -2482,8 +2531,13 @@
       <c r="U33" s="10"/>
       <c r="V33" s="10"/>
       <c r="W33" s="10"/>
-      <c r="X33" s="11"/>
-      <c r="Y33" s="9"/>
+      <c r="X33" s="11">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="Y33" s="9">
+        <v>0</v>
+      </c>
       <c r="Z33" s="28"/>
     </row>
     <row r="34" spans="1:26">
@@ -2520,8 +2574,13 @@
       <c r="U34" s="10"/>
       <c r="V34" s="10"/>
       <c r="W34" s="10"/>
-      <c r="X34" s="11"/>
-      <c r="Y34" s="9"/>
+      <c r="X34" s="11">
+        <f t="shared" si="1"/>
+        <v>6</v>
+      </c>
+      <c r="Y34" s="9">
+        <v>0</v>
+      </c>
       <c r="Z34" s="28"/>
     </row>
     <row r="35" spans="1:26">
@@ -2538,28 +2597,37 @@
         <v>44</v>
       </c>
       <c r="G35" s="9">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="H35" s="10"/>
       <c r="I35" s="10"/>
       <c r="J35" s="10"/>
       <c r="K35" s="10"/>
       <c r="L35" s="10"/>
-      <c r="M35" s="10"/>
-      <c r="N35" s="10">
-        <v>3</v>
-      </c>
+      <c r="M35" s="10">
+        <v>6</v>
+      </c>
+      <c r="N35" s="10"/>
       <c r="O35" s="10"/>
       <c r="P35" s="10"/>
       <c r="Q35" s="10"/>
       <c r="R35" s="10"/>
-      <c r="S35" s="10"/>
-      <c r="T35" s="10"/>
+      <c r="S35" s="10">
+        <v>6</v>
+      </c>
+      <c r="T35" s="10">
+        <v>4</v>
+      </c>
       <c r="U35" s="10"/>
       <c r="V35" s="10"/>
       <c r="W35" s="10"/>
-      <c r="X35" s="11"/>
-      <c r="Y35" s="9"/>
+      <c r="X35" s="11">
+        <f t="shared" si="1"/>
+        <v>16</v>
+      </c>
+      <c r="Y35" s="9">
+        <v>0</v>
+      </c>
       <c r="Z35" s="28"/>
     </row>
     <row r="36" spans="1:26">
@@ -2567,31 +2635,44 @@
         <v>92</v>
       </c>
       <c r="B36" s="7"/>
-      <c r="C36" s="8" t="s">
+      <c r="C36" s="8"/>
+      <c r="D36" s="8" t="s">
         <v>93</v>
       </c>
-      <c r="D36" s="8"/>
       <c r="E36" s="8"/>
-      <c r="F36" s="8"/>
-      <c r="G36" s="9"/>
+      <c r="F36" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="G36" s="9">
+        <v>5</v>
+      </c>
       <c r="H36" s="10"/>
       <c r="I36" s="10"/>
       <c r="J36" s="10"/>
       <c r="K36" s="10"/>
       <c r="L36" s="10"/>
       <c r="M36" s="10"/>
-      <c r="N36" s="10"/>
+      <c r="N36" s="10">
+        <v>3</v>
+      </c>
       <c r="O36" s="10"/>
       <c r="P36" s="10"/>
       <c r="Q36" s="10"/>
-      <c r="R36" s="10"/>
+      <c r="R36" s="10">
+        <v>1</v>
+      </c>
       <c r="S36" s="10"/>
       <c r="T36" s="10"/>
       <c r="U36" s="10"/>
       <c r="V36" s="10"/>
       <c r="W36" s="10"/>
-      <c r="X36" s="11"/>
-      <c r="Y36" s="9"/>
+      <c r="X36" s="11">
+        <f t="shared" si="1"/>
+        <v>4</v>
+      </c>
+      <c r="Y36" s="9">
+        <v>0</v>
+      </c>
       <c r="Z36" s="28"/>
     </row>
     <row r="37" spans="1:26">
@@ -2599,22 +2680,16 @@
         <v>94</v>
       </c>
       <c r="B37" s="7"/>
-      <c r="C37" s="8"/>
-      <c r="D37" s="8" t="s">
+      <c r="C37" s="8" t="s">
         <v>95</v>
       </c>
+      <c r="D37" s="8"/>
       <c r="E37" s="8"/>
-      <c r="F37" s="8" t="s">
-        <v>96</v>
-      </c>
-      <c r="G37" s="9">
-        <v>5</v>
-      </c>
+      <c r="F37" s="8"/>
+      <c r="G37" s="9"/>
       <c r="H37" s="10"/>
       <c r="I37" s="10"/>
-      <c r="J37" s="10">
-        <v>7</v>
-      </c>
+      <c r="J37" s="10"/>
       <c r="K37" s="10"/>
       <c r="L37" s="10"/>
       <c r="M37" s="10"/>
@@ -2628,32 +2703,35 @@
       <c r="U37" s="10"/>
       <c r="V37" s="10"/>
       <c r="W37" s="10"/>
-      <c r="X37" s="11"/>
+      <c r="X37" s="11">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
       <c r="Y37" s="9"/>
       <c r="Z37" s="28"/>
     </row>
     <row r="38" spans="1:26">
       <c r="A38" s="6" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B38" s="7"/>
       <c r="C38" s="8"/>
       <c r="D38" s="8" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="E38" s="8"/>
       <c r="F38" s="8" t="s">
-        <v>25</v>
+        <v>98</v>
       </c>
       <c r="G38" s="9">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="H38" s="10"/>
       <c r="I38" s="10"/>
-      <c r="J38" s="10"/>
-      <c r="K38" s="10">
+      <c r="J38" s="10">
         <v>7</v>
       </c>
+      <c r="K38" s="10"/>
       <c r="L38" s="10"/>
       <c r="M38" s="10"/>
       <c r="N38" s="10"/>
@@ -2666,8 +2744,13 @@
       <c r="U38" s="10"/>
       <c r="V38" s="10"/>
       <c r="W38" s="10"/>
-      <c r="X38" s="11"/>
-      <c r="Y38" s="9"/>
+      <c r="X38" s="11">
+        <f t="shared" si="1"/>
+        <v>7</v>
+      </c>
+      <c r="Y38" s="9">
+        <v>0</v>
+      </c>
       <c r="Z38" s="28"/>
     </row>
     <row r="39" spans="1:26">
@@ -2684,15 +2767,15 @@
         <v>25</v>
       </c>
       <c r="G39" s="9">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="H39" s="10"/>
       <c r="I39" s="10"/>
       <c r="J39" s="10"/>
-      <c r="K39" s="10"/>
-      <c r="L39" s="10">
-        <v>5</v>
-      </c>
+      <c r="K39" s="10">
+        <v>7</v>
+      </c>
+      <c r="L39" s="10"/>
       <c r="M39" s="10"/>
       <c r="N39" s="10"/>
       <c r="O39" s="10"/>
@@ -2705,14 +2788,13 @@
       <c r="V39" s="10"/>
       <c r="W39" s="10"/>
       <c r="X39" s="11">
-        <f>SUM(H39:W39)</f>
-        <v>5</v>
-      </c>
-      <c r="Y39" s="9"/>
-      <c r="Z39" s="28">
-        <f>G39-X39-Y39</f>
-        <v>10</v>
-      </c>
+        <f t="shared" si="1"/>
+        <v>7</v>
+      </c>
+      <c r="Y39" s="9">
+        <v>0</v>
+      </c>
+      <c r="Z39" s="28"/>
     </row>
     <row r="40" spans="1:26">
       <c r="A40" s="6" t="s">
@@ -2725,7 +2807,7 @@
       </c>
       <c r="E40" s="8"/>
       <c r="F40" s="8" t="s">
-        <v>103</v>
+        <v>25</v>
       </c>
       <c r="G40" s="9">
         <v>15</v>
@@ -2734,47 +2816,55 @@
       <c r="I40" s="10"/>
       <c r="J40" s="10"/>
       <c r="K40" s="10"/>
-      <c r="L40" s="10"/>
-      <c r="M40" s="10">
+      <c r="L40" s="10">
         <v>5</v>
       </c>
-      <c r="N40" s="10">
-        <v>5</v>
-      </c>
+      <c r="M40" s="10"/>
+      <c r="N40" s="10"/>
       <c r="O40" s="10"/>
       <c r="P40" s="10"/>
       <c r="Q40" s="10"/>
-      <c r="R40" s="10"/>
-      <c r="S40" s="10"/>
-      <c r="T40" s="10"/>
-      <c r="U40" s="10"/>
-      <c r="V40" s="10"/>
+      <c r="R40" s="10">
+        <v>2</v>
+      </c>
+      <c r="S40" s="10">
+        <v>3</v>
+      </c>
+      <c r="T40" s="10">
+        <v>5</v>
+      </c>
+      <c r="U40" s="10">
+        <v>5</v>
+      </c>
+      <c r="V40" s="10">
+        <v>5</v>
+      </c>
       <c r="W40" s="10"/>
       <c r="X40" s="11">
-        <f>SUM(H40:W40)</f>
-        <v>10</v>
+        <f t="shared" si="1"/>
+        <v>25</v>
       </c>
       <c r="Y40" s="9"/>
       <c r="Z40" s="28">
         <f>G40-X40-Y40</f>
-        <v>5</v>
+        <v>-10</v>
       </c>
     </row>
     <row r="41" spans="1:26">
       <c r="A41" s="6" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B41" s="7"/>
       <c r="C41" s="8"/>
       <c r="D41" s="8" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="E41" s="8"/>
       <c r="F41" s="8" t="s">
-        <v>37</v>
+        <v>105</v>
       </c>
       <c r="G41" s="9">
-        <v>5</v>
+        <v>25</v>
       </c>
       <c r="H41" s="10"/>
       <c r="I41" s="10"/>
@@ -2784,24 +2874,38 @@
       <c r="M41" s="10">
         <v>5</v>
       </c>
-      <c r="N41" s="10"/>
+      <c r="N41" s="10">
+        <v>5</v>
+      </c>
       <c r="O41" s="10"/>
-      <c r="P41" s="10"/>
+      <c r="P41" s="10">
+        <v>10</v>
+      </c>
       <c r="Q41" s="10"/>
       <c r="R41" s="10"/>
       <c r="S41" s="10"/>
-      <c r="T41" s="10"/>
-      <c r="U41" s="10"/>
-      <c r="V41" s="10"/>
-      <c r="W41" s="10"/>
+      <c r="T41" s="10">
+        <v>5</v>
+      </c>
+      <c r="U41" s="10">
+        <v>5</v>
+      </c>
+      <c r="V41" s="10">
+        <v>5</v>
+      </c>
+      <c r="W41" s="10">
+        <v>5</v>
+      </c>
       <c r="X41" s="11">
-        <f>SUM(H41:W41)</f>
-        <v>5</v>
-      </c>
-      <c r="Y41" s="9"/>
+        <f t="shared" si="1"/>
+        <v>40</v>
+      </c>
+      <c r="Y41" s="9">
+        <v>0</v>
+      </c>
       <c r="Z41" s="28">
         <f>G41-X41-Y41</f>
-        <v>0</v>
+        <v>-15</v>
       </c>
     </row>
     <row r="42" spans="1:26">
@@ -2811,20 +2915,28 @@
       <c r="B42" s="7"/>
       <c r="C42" s="8"/>
       <c r="D42" s="8" t="s">
-        <v>50</v>
+        <v>107</v>
       </c>
       <c r="E42" s="8"/>
-      <c r="F42" s="8"/>
-      <c r="G42" s="9"/>
+      <c r="F42" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="G42" s="9">
+        <v>5</v>
+      </c>
       <c r="H42" s="10"/>
       <c r="I42" s="10"/>
       <c r="J42" s="10"/>
       <c r="K42" s="10"/>
       <c r="L42" s="10"/>
-      <c r="M42" s="10"/>
+      <c r="M42" s="10">
+        <v>5</v>
+      </c>
       <c r="N42" s="10"/>
       <c r="O42" s="10"/>
-      <c r="P42" s="10"/>
+      <c r="P42" s="10">
+        <v>6</v>
+      </c>
       <c r="Q42" s="10"/>
       <c r="R42" s="10"/>
       <c r="S42" s="10"/>
@@ -2834,23 +2946,25 @@
       <c r="W42" s="10"/>
       <c r="X42" s="11">
         <f>SUM(H42:W42)</f>
-        <v>0</v>
-      </c>
-      <c r="Y42" s="9"/>
+        <v>11</v>
+      </c>
+      <c r="Y42" s="9">
+        <v>0</v>
+      </c>
       <c r="Z42" s="28">
         <f>G42-X42-Y42</f>
-        <v>0</v>
+        <v>-6</v>
       </c>
     </row>
     <row r="43" spans="1:26">
       <c r="A43" s="6" t="s">
-        <v>107</v>
-      </c>
-      <c r="B43" s="7" t="s">
         <v>108</v>
       </c>
+      <c r="B43" s="7"/>
       <c r="C43" s="8"/>
-      <c r="D43" s="8"/>
+      <c r="D43" s="8" t="s">
+        <v>50</v>
+      </c>
       <c r="E43" s="8"/>
       <c r="F43" s="8"/>
       <c r="G43" s="9"/>
@@ -2871,12 +2985,12 @@
       <c r="V43" s="10"/>
       <c r="W43" s="10"/>
       <c r="X43" s="11">
-        <f t="shared" si="4"/>
+        <f>SUM(H43:W43)</f>
         <v>0</v>
       </c>
       <c r="Y43" s="9"/>
       <c r="Z43" s="28">
-        <f t="shared" si="0"/>
+        <f>G43-X43-Y43</f>
         <v>0</v>
       </c>
     </row>
@@ -2884,32 +2998,22 @@
       <c r="A44" s="6" t="s">
         <v>109</v>
       </c>
-      <c r="B44" s="7"/>
-      <c r="C44" s="8" t="s">
+      <c r="B44" s="7" t="s">
         <v>110</v>
       </c>
+      <c r="C44" s="8"/>
       <c r="D44" s="8"/>
       <c r="E44" s="8"/>
-      <c r="F44" s="8" t="s">
-        <v>37</v>
-      </c>
-      <c r="G44" s="9">
-        <v>20</v>
-      </c>
+      <c r="F44" s="8"/>
+      <c r="G44" s="9"/>
       <c r="H44" s="10"/>
       <c r="I44" s="10"/>
       <c r="J44" s="10"/>
       <c r="K44" s="10"/>
-      <c r="L44" s="10">
-        <v>5</v>
-      </c>
-      <c r="M44" s="10">
-        <v>5</v>
-      </c>
+      <c r="L44" s="10"/>
+      <c r="M44" s="10"/>
       <c r="N44" s="10"/>
-      <c r="O44" s="10">
-        <v>5</v>
-      </c>
+      <c r="O44" s="10"/>
       <c r="P44" s="10"/>
       <c r="Q44" s="10"/>
       <c r="R44" s="10"/>
@@ -2919,13 +3023,13 @@
       <c r="V44" s="10"/>
       <c r="W44" s="10"/>
       <c r="X44" s="11">
-        <f t="shared" si="4"/>
-        <v>15</v>
+        <f t="shared" ref="X26:X62" si="2">SUM(H44:W44)</f>
+        <v>0</v>
       </c>
       <c r="Y44" s="9"/>
       <c r="Z44" s="28">
-        <f t="shared" si="0"/>
-        <v>5</v>
+        <f>G44-X44-Y44</f>
+        <v>0</v>
       </c>
     </row>
     <row r="45" spans="1:26">
@@ -2942,17 +3046,25 @@
         <v>37</v>
       </c>
       <c r="G45" s="9">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="H45" s="10"/>
       <c r="I45" s="10"/>
       <c r="J45" s="10"/>
       <c r="K45" s="10"/>
-      <c r="L45" s="10"/>
-      <c r="M45" s="10"/>
+      <c r="L45" s="10">
+        <v>5</v>
+      </c>
+      <c r="M45" s="10">
+        <v>5</v>
+      </c>
       <c r="N45" s="10"/>
-      <c r="O45" s="10"/>
-      <c r="P45" s="10"/>
+      <c r="O45" s="10">
+        <v>5</v>
+      </c>
+      <c r="P45" s="10">
+        <v>5</v>
+      </c>
       <c r="Q45" s="10"/>
       <c r="R45" s="10"/>
       <c r="S45" s="10"/>
@@ -2961,13 +3073,13 @@
       <c r="V45" s="10"/>
       <c r="W45" s="10"/>
       <c r="X45" s="11">
-        <f t="shared" si="4"/>
-        <v>0</v>
+        <f t="shared" si="2"/>
+        <v>20</v>
       </c>
       <c r="Y45" s="9"/>
       <c r="Z45" s="28">
-        <f t="shared" si="0"/>
-        <v>10</v>
+        <f>G45-X45-Y45</f>
+        <v>0</v>
       </c>
     </row>
     <row r="46" spans="1:26">
@@ -2981,10 +3093,10 @@
       <c r="D46" s="8"/>
       <c r="E46" s="8"/>
       <c r="F46" s="8" t="s">
-        <v>31</v>
+        <v>115</v>
       </c>
       <c r="G46" s="9">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="H46" s="10"/>
       <c r="I46" s="10"/>
@@ -2998,32 +3110,37 @@
       <c r="Q46" s="10"/>
       <c r="R46" s="10"/>
       <c r="S46" s="10"/>
-      <c r="T46" s="10"/>
-      <c r="U46" s="10"/>
+      <c r="T46" s="10">
+        <v>10</v>
+      </c>
+      <c r="U46" s="10">
+        <v>10</v>
+      </c>
       <c r="V46" s="10"/>
       <c r="W46" s="10"/>
       <c r="X46" s="11">
-        <f t="shared" si="4"/>
-        <v>0</v>
+        <f t="shared" si="2"/>
+        <v>20</v>
       </c>
       <c r="Y46" s="9"/>
-      <c r="Z46" s="28">
-        <f t="shared" si="0"/>
-        <v>30</v>
-      </c>
+      <c r="Z46" s="28"/>
     </row>
     <row r="47" spans="1:26">
       <c r="A47" s="6" t="s">
-        <v>115</v>
-      </c>
-      <c r="B47" s="7" t="s">
         <v>116</v>
       </c>
-      <c r="C47" s="8"/>
+      <c r="B47" s="7"/>
+      <c r="C47" s="8" t="s">
+        <v>117</v>
+      </c>
       <c r="D47" s="8"/>
       <c r="E47" s="8"/>
-      <c r="F47" s="8"/>
-      <c r="G47" s="9"/>
+      <c r="F47" s="8" t="s">
+        <v>118</v>
+      </c>
+      <c r="G47" s="9">
+        <v>10</v>
+      </c>
       <c r="H47" s="10"/>
       <c r="I47" s="10"/>
       <c r="J47" s="10"/>
@@ -3031,8 +3148,12 @@
       <c r="L47" s="10"/>
       <c r="M47" s="10"/>
       <c r="N47" s="10"/>
-      <c r="O47" s="10"/>
-      <c r="P47" s="10"/>
+      <c r="O47" s="10">
+        <v>5</v>
+      </c>
+      <c r="P47" s="10">
+        <v>5</v>
+      </c>
       <c r="Q47" s="10"/>
       <c r="R47" s="10"/>
       <c r="S47" s="10"/>
@@ -3041,30 +3162,30 @@
       <c r="V47" s="10"/>
       <c r="W47" s="10"/>
       <c r="X47" s="11">
-        <f t="shared" si="4"/>
-        <v>0</v>
+        <f t="shared" si="2"/>
+        <v>10</v>
       </c>
       <c r="Y47" s="9"/>
       <c r="Z47" s="28">
-        <f t="shared" si="0"/>
+        <f>G47-X47-Y47</f>
         <v>0</v>
       </c>
     </row>
     <row r="48" spans="1:26">
       <c r="A48" s="6" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B48" s="7"/>
       <c r="C48" s="8" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="D48" s="8"/>
       <c r="E48" s="8"/>
       <c r="F48" s="8" t="s">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="G48" s="9">
-        <v>4</v>
+        <v>30</v>
       </c>
       <c r="H48" s="10"/>
       <c r="I48" s="10"/>
@@ -3073,41 +3194,49 @@
       <c r="L48" s="10"/>
       <c r="M48" s="10"/>
       <c r="N48" s="10"/>
-      <c r="O48" s="10"/>
-      <c r="P48" s="10"/>
-      <c r="Q48" s="10"/>
+      <c r="O48" s="10">
+        <v>5</v>
+      </c>
+      <c r="P48" s="10">
+        <v>5</v>
+      </c>
+      <c r="Q48" s="10">
+        <v>5</v>
+      </c>
       <c r="R48" s="10"/>
       <c r="S48" s="10"/>
       <c r="T48" s="10"/>
-      <c r="U48" s="10"/>
-      <c r="V48" s="10"/>
+      <c r="U48" s="10">
+        <v>6</v>
+      </c>
+      <c r="V48" s="10">
+        <v>2</v>
+      </c>
       <c r="W48" s="10"/>
       <c r="X48" s="11">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="Y48" s="9"/>
+        <f t="shared" si="2"/>
+        <v>23</v>
+      </c>
+      <c r="Y48" s="9">
+        <v>0</v>
+      </c>
       <c r="Z48" s="28">
-        <f t="shared" si="0"/>
-        <v>4</v>
+        <f>G48-X48-Y48</f>
+        <v>7</v>
       </c>
     </row>
     <row r="49" spans="1:26">
       <c r="A49" s="6" t="s">
-        <v>119</v>
-      </c>
-      <c r="B49" s="7"/>
-      <c r="C49" s="8" t="s">
-        <v>120</v>
-      </c>
+        <v>121</v>
+      </c>
+      <c r="B49" s="7" t="s">
+        <v>122</v>
+      </c>
+      <c r="C49" s="8"/>
       <c r="D49" s="8"/>
       <c r="E49" s="8"/>
-      <c r="F49" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="G49" s="9">
-        <v>15</v>
-      </c>
+      <c r="F49" s="8"/>
+      <c r="G49" s="9"/>
       <c r="H49" s="10"/>
       <c r="I49" s="10"/>
       <c r="J49" s="10"/>
@@ -3125,30 +3254,30 @@
       <c r="V49" s="10"/>
       <c r="W49" s="10"/>
       <c r="X49" s="11">
-        <f t="shared" si="4"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="Y49" s="9"/>
       <c r="Z49" s="28">
-        <f t="shared" si="0"/>
-        <v>15</v>
+        <f>G49-X49-Y49</f>
+        <v>0</v>
       </c>
     </row>
     <row r="50" spans="1:26">
       <c r="A50" s="6" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="B50" s="7"/>
       <c r="C50" s="8" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="D50" s="8"/>
       <c r="E50" s="8"/>
       <c r="F50" s="8" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
       <c r="G50" s="9">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H50" s="10"/>
       <c r="I50" s="10"/>
@@ -3159,7 +3288,9 @@
       <c r="N50" s="10"/>
       <c r="O50" s="10"/>
       <c r="P50" s="10"/>
-      <c r="Q50" s="10"/>
+      <c r="Q50" s="10">
+        <v>5</v>
+      </c>
       <c r="R50" s="10"/>
       <c r="S50" s="10"/>
       <c r="T50" s="10"/>
@@ -3167,30 +3298,32 @@
       <c r="V50" s="10"/>
       <c r="W50" s="10"/>
       <c r="X50" s="11">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="Y50" s="9"/>
+        <f t="shared" si="2"/>
+        <v>5</v>
+      </c>
+      <c r="Y50" s="9">
+        <v>0</v>
+      </c>
       <c r="Z50" s="28">
-        <f t="shared" si="0"/>
-        <v>2</v>
+        <f>G50-X50-Y50</f>
+        <v>-1</v>
       </c>
     </row>
     <row r="51" spans="1:26">
       <c r="A51" s="6" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="B51" s="7"/>
       <c r="C51" s="8" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="D51" s="8"/>
       <c r="E51" s="8"/>
       <c r="F51" s="8" t="s">
-        <v>37</v>
+        <v>31</v>
       </c>
       <c r="G51" s="9">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="H51" s="10"/>
       <c r="I51" s="10"/>
@@ -3206,33 +3339,37 @@
       <c r="S51" s="10"/>
       <c r="T51" s="10"/>
       <c r="U51" s="10"/>
-      <c r="V51" s="10"/>
+      <c r="V51" s="10">
+        <v>20</v>
+      </c>
       <c r="W51" s="10"/>
       <c r="X51" s="11">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="Y51" s="9"/>
+        <f t="shared" si="2"/>
+        <v>20</v>
+      </c>
+      <c r="Y51" s="9">
+        <v>0</v>
+      </c>
       <c r="Z51" s="28">
-        <f t="shared" si="0"/>
-        <v>6</v>
+        <f>G51-X51-Y51</f>
+        <v>-5</v>
       </c>
     </row>
     <row r="52" spans="1:26">
       <c r="A52" s="6" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="B52" s="7"/>
       <c r="C52" s="8" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="D52" s="8"/>
       <c r="E52" s="8"/>
       <c r="F52" s="8" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="G52" s="9">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H52" s="10"/>
       <c r="I52" s="10"/>
@@ -3248,33 +3385,37 @@
       <c r="S52" s="10"/>
       <c r="T52" s="10"/>
       <c r="U52" s="10"/>
-      <c r="V52" s="10"/>
+      <c r="V52" s="26">
+        <v>2</v>
+      </c>
       <c r="W52" s="10"/>
       <c r="X52" s="11">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="Y52" s="9"/>
+        <f t="shared" si="2"/>
+        <v>2</v>
+      </c>
+      <c r="Y52" s="9">
+        <v>0</v>
+      </c>
       <c r="Z52" s="28">
-        <f t="shared" si="0"/>
-        <v>3</v>
+        <f>G52-X52-Y52</f>
+        <v>0</v>
       </c>
     </row>
     <row r="53" spans="1:26">
       <c r="A53" s="6" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B53" s="7"/>
       <c r="C53" s="8" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="D53" s="8"/>
       <c r="E53" s="8"/>
       <c r="F53" s="8" t="s">
-        <v>31</v>
+        <v>42</v>
       </c>
       <c r="G53" s="9">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="H53" s="10"/>
       <c r="I53" s="10"/>
@@ -3289,34 +3430,40 @@
       <c r="R53" s="10"/>
       <c r="S53" s="10"/>
       <c r="T53" s="10"/>
-      <c r="U53" s="10"/>
-      <c r="V53" s="10"/>
+      <c r="U53" s="10">
+        <v>3</v>
+      </c>
+      <c r="V53" s="10">
+        <v>3</v>
+      </c>
       <c r="W53" s="10"/>
       <c r="X53" s="11">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="Y53" s="9"/>
+        <f t="shared" si="2"/>
+        <v>6</v>
+      </c>
+      <c r="Y53" s="9">
+        <v>0</v>
+      </c>
       <c r="Z53" s="28">
-        <f t="shared" si="0"/>
-        <v>2</v>
+        <f>G53-X53-Y53</f>
+        <v>0</v>
       </c>
     </row>
     <row r="54" spans="1:26">
       <c r="A54" s="6" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="B54" s="7"/>
       <c r="C54" s="8" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="D54" s="8"/>
       <c r="E54" s="8"/>
       <c r="F54" s="8" t="s">
-        <v>31</v>
+        <v>44</v>
       </c>
       <c r="G54" s="9">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="H54" s="10"/>
       <c r="I54" s="10"/>
@@ -3326,34 +3473,44 @@
       <c r="M54" s="10"/>
       <c r="N54" s="10"/>
       <c r="O54" s="10"/>
-      <c r="P54" s="10">
-        <v>2</v>
-      </c>
+      <c r="P54" s="10"/>
       <c r="Q54" s="10"/>
       <c r="R54" s="10"/>
       <c r="S54" s="10"/>
       <c r="T54" s="10"/>
       <c r="U54" s="10"/>
-      <c r="V54" s="10"/>
+      <c r="V54" s="10">
+        <v>3</v>
+      </c>
       <c r="W54" s="10"/>
       <c r="X54" s="11">
-        <f t="shared" si="4"/>
-        <v>2</v>
-      </c>
-      <c r="Y54" s="9"/>
+        <f t="shared" si="2"/>
+        <v>3</v>
+      </c>
+      <c r="Y54" s="9">
+        <v>0</v>
+      </c>
       <c r="Z54" s="28">
-        <f t="shared" si="0"/>
-        <v>6</v>
+        <f>G54-X54-Y54</f>
+        <v>0</v>
       </c>
     </row>
     <row r="55" spans="1:26">
-      <c r="A55" s="6"/>
+      <c r="A55" s="6" t="s">
+        <v>133</v>
+      </c>
       <c r="B55" s="7"/>
-      <c r="C55" s="8"/>
+      <c r="C55" s="8" t="s">
+        <v>134</v>
+      </c>
       <c r="D55" s="8"/>
       <c r="E55" s="8"/>
-      <c r="F55" s="8"/>
-      <c r="G55" s="9"/>
+      <c r="F55" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="G55" s="9">
+        <v>2</v>
+      </c>
       <c r="H55" s="10"/>
       <c r="I55" s="10"/>
       <c r="J55" s="10"/>
@@ -3363,191 +3520,215 @@
       <c r="N55" s="10"/>
       <c r="O55" s="10"/>
       <c r="P55" s="10"/>
-      <c r="Q55" s="10"/>
+      <c r="Q55" s="10">
+        <v>2</v>
+      </c>
       <c r="R55" s="10"/>
       <c r="S55" s="10"/>
-      <c r="T55" s="10"/>
-      <c r="U55" s="10"/>
+      <c r="T55" s="10">
+        <v>1</v>
+      </c>
+      <c r="U55" s="10">
+        <v>2</v>
+      </c>
       <c r="V55" s="10"/>
       <c r="W55" s="10"/>
       <c r="X55" s="11">
-        <f t="shared" si="4"/>
-        <v>0</v>
+        <f t="shared" si="2"/>
+        <v>5</v>
       </c>
       <c r="Y55" s="9"/>
       <c r="Z55" s="28">
-        <f t="shared" si="0"/>
-        <v>0</v>
+        <f>G55-X55-Y55</f>
+        <v>-3</v>
       </c>
     </row>
     <row r="56" spans="1:26">
-      <c r="A56" s="16" t="s">
-        <v>131</v>
-      </c>
-      <c r="B56" s="13" t="s">
-        <v>132</v>
-      </c>
-      <c r="C56" s="12"/>
-      <c r="D56" s="12"/>
-      <c r="E56" s="12"/>
-      <c r="F56" s="8"/>
-      <c r="G56" s="8">
+      <c r="A56" s="6" t="s">
+        <v>135</v>
+      </c>
+      <c r="B56" s="7"/>
+      <c r="C56" s="8" t="s">
+        <v>136</v>
+      </c>
+      <c r="D56" s="8"/>
+      <c r="E56" s="8"/>
+      <c r="F56" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="G56" s="9">
+        <v>8</v>
+      </c>
+      <c r="H56" s="10"/>
+      <c r="I56" s="10"/>
+      <c r="J56" s="10"/>
+      <c r="K56" s="10"/>
+      <c r="L56" s="10"/>
+      <c r="M56" s="10"/>
+      <c r="N56" s="10"/>
+      <c r="O56" s="10"/>
+      <c r="P56" s="10">
+        <v>2</v>
+      </c>
+      <c r="Q56" s="10">
+        <v>2</v>
+      </c>
+      <c r="R56" s="10"/>
+      <c r="S56" s="10"/>
+      <c r="T56" s="10"/>
+      <c r="U56" s="10"/>
+      <c r="V56" s="10">
+        <v>5</v>
+      </c>
+      <c r="W56" s="10"/>
+      <c r="X56" s="11">
+        <f t="shared" si="2"/>
+        <v>9</v>
+      </c>
+      <c r="Y56" s="9">
+        <v>0</v>
+      </c>
+      <c r="Z56" s="28">
+        <f>G56-X56-Y56</f>
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="57" spans="1:26">
+      <c r="A57" s="6"/>
+      <c r="B57" s="7"/>
+      <c r="C57" s="8"/>
+      <c r="D57" s="8"/>
+      <c r="E57" s="8"/>
+      <c r="F57" s="8"/>
+      <c r="G57" s="9"/>
+      <c r="H57" s="10"/>
+      <c r="I57" s="10"/>
+      <c r="J57" s="10"/>
+      <c r="K57" s="10"/>
+      <c r="L57" s="10"/>
+      <c r="M57" s="10"/>
+      <c r="N57" s="10"/>
+      <c r="O57" s="10"/>
+      <c r="P57" s="10"/>
+      <c r="Q57" s="10"/>
+      <c r="R57" s="10"/>
+      <c r="S57" s="10"/>
+      <c r="T57" s="10"/>
+      <c r="U57" s="10"/>
+      <c r="V57" s="10"/>
+      <c r="W57" s="10"/>
+      <c r="X57" s="11">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="Y57" s="9"/>
+      <c r="Z57" s="28">
+        <f>G57-X57-Y57</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58" spans="1:26">
+      <c r="A58" s="16" t="s">
+        <v>137</v>
+      </c>
+      <c r="B58" s="13" t="s">
+        <v>138</v>
+      </c>
+      <c r="C58" s="12"/>
+      <c r="D58" s="12"/>
+      <c r="E58" s="12"/>
+      <c r="F58" s="8"/>
+      <c r="G58" s="8">
         <v>30</v>
       </c>
-      <c r="H56" s="15"/>
-      <c r="I56" s="15"/>
-      <c r="J56" s="15"/>
-      <c r="K56" s="15"/>
-      <c r="L56" s="15"/>
-      <c r="M56" s="15"/>
-      <c r="N56" s="15"/>
-      <c r="O56" s="15"/>
-      <c r="P56" s="15"/>
-      <c r="Q56" s="15"/>
-      <c r="R56" s="15"/>
-      <c r="S56" s="15"/>
-      <c r="T56" s="15"/>
-      <c r="U56" s="15"/>
-      <c r="V56" s="15"/>
-      <c r="W56" s="15"/>
-      <c r="X56" s="11">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="Y56" s="9"/>
-      <c r="Z56" s="28">
-        <f t="shared" si="0"/>
-        <v>30</v>
-      </c>
-    </row>
-    <row r="57" spans="1:26">
-      <c r="A57" s="16" t="s">
-        <v>133</v>
-      </c>
-      <c r="B57" s="13" t="s">
-        <v>134</v>
-      </c>
-      <c r="C57" s="12"/>
-      <c r="D57" s="12"/>
-      <c r="E57" s="12"/>
-      <c r="F57" s="8"/>
-      <c r="G57" s="8"/>
-      <c r="H57" s="15"/>
-      <c r="I57" s="15"/>
-      <c r="J57" s="15"/>
-      <c r="K57" s="15"/>
-      <c r="L57" s="15"/>
-      <c r="M57" s="15"/>
-      <c r="N57" s="15"/>
-      <c r="O57" s="15"/>
-      <c r="P57" s="15"/>
-      <c r="Q57" s="15"/>
-      <c r="R57" s="15"/>
-      <c r="S57" s="15"/>
-      <c r="T57" s="15"/>
-      <c r="U57" s="15"/>
-      <c r="V57" s="15"/>
-      <c r="W57" s="15"/>
-      <c r="X57" s="11">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="Y57" s="14"/>
-      <c r="Z57" s="28">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="58" spans="1:26">
-      <c r="A58" s="17"/>
-      <c r="B58" s="18"/>
-      <c r="C58" s="19" t="s">
-        <v>135</v>
-      </c>
-      <c r="D58" s="19"/>
-      <c r="E58" s="19"/>
-      <c r="F58" s="8" t="s">
+      <c r="H58" s="15"/>
+      <c r="I58" s="15"/>
+      <c r="J58" s="15"/>
+      <c r="K58" s="15"/>
+      <c r="L58" s="15"/>
+      <c r="M58" s="15"/>
+      <c r="N58" s="15"/>
+      <c r="O58" s="15"/>
+      <c r="P58" s="15"/>
+      <c r="Q58" s="15"/>
+      <c r="R58" s="15"/>
+      <c r="S58" s="15"/>
+      <c r="T58" s="15">
+        <v>5</v>
+      </c>
+      <c r="U58" s="15"/>
+      <c r="V58" s="15"/>
+      <c r="W58" s="15"/>
+      <c r="X58" s="11">
+        <f t="shared" si="2"/>
+        <v>5</v>
+      </c>
+      <c r="Y58" s="9">
+        <v>0</v>
+      </c>
+      <c r="Z58" s="28">
+        <f>G58-X58-Y58</f>
         <v>25</v>
       </c>
-      <c r="G58" s="8">
-        <v>4</v>
-      </c>
-      <c r="H58" s="21"/>
-      <c r="I58" s="21"/>
-      <c r="J58" s="21"/>
-      <c r="K58" s="21"/>
-      <c r="L58" s="21"/>
-      <c r="M58" s="21"/>
-      <c r="N58" s="21"/>
-      <c r="O58" s="21"/>
-      <c r="P58" s="21"/>
-      <c r="Q58" s="21"/>
-      <c r="R58" s="21"/>
-      <c r="S58" s="21"/>
-      <c r="T58" s="21"/>
-      <c r="U58" s="21"/>
-      <c r="V58" s="21"/>
-      <c r="W58" s="21"/>
-      <c r="X58" s="11">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="Y58" s="20"/>
-      <c r="Z58" s="28">
-        <f t="shared" si="0"/>
-        <v>4</v>
-      </c>
     </row>
     <row r="59" spans="1:26">
-      <c r="A59" s="17"/>
-      <c r="B59" s="18"/>
-      <c r="C59" s="19" t="s">
-        <v>136</v>
-      </c>
-      <c r="D59" s="19"/>
-      <c r="E59" s="19"/>
-      <c r="F59" s="8" t="s">
-        <v>25</v>
-      </c>
-      <c r="G59" s="8">
-        <v>16</v>
-      </c>
-      <c r="H59" s="21"/>
-      <c r="I59" s="21"/>
-      <c r="J59" s="21"/>
-      <c r="K59" s="21"/>
-      <c r="L59" s="21"/>
-      <c r="M59" s="21"/>
-      <c r="N59" s="21"/>
-      <c r="O59" s="21"/>
-      <c r="P59" s="21"/>
-      <c r="Q59" s="21"/>
-      <c r="R59" s="21"/>
-      <c r="S59" s="21"/>
-      <c r="T59" s="21"/>
-      <c r="U59" s="21"/>
-      <c r="V59" s="21"/>
-      <c r="W59" s="21"/>
+      <c r="A59" s="16" t="s">
+        <v>139</v>
+      </c>
+      <c r="B59" s="13" t="s">
+        <v>140</v>
+      </c>
+      <c r="C59" s="12"/>
+      <c r="D59" s="12"/>
+      <c r="E59" s="12"/>
+      <c r="F59" s="8"/>
+      <c r="G59" s="8"/>
+      <c r="H59" s="15"/>
+      <c r="I59" s="15"/>
+      <c r="J59" s="15"/>
+      <c r="K59" s="15"/>
+      <c r="L59" s="15"/>
+      <c r="M59" s="15"/>
+      <c r="N59" s="15"/>
+      <c r="O59" s="15"/>
+      <c r="P59" s="15"/>
+      <c r="Q59" s="15"/>
+      <c r="R59" s="15"/>
+      <c r="S59" s="15"/>
+      <c r="T59" s="15"/>
+      <c r="U59" s="15"/>
+      <c r="V59" s="15"/>
+      <c r="W59" s="15"/>
       <c r="X59" s="11">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="Y59" s="20"/>
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="Y59" s="14"/>
       <c r="Z59" s="28">
-        <f t="shared" si="0"/>
-        <v>16</v>
-      </c>
-    </row>
-    <row r="60" spans="1:26" ht="12.6" thickBot="1">
+        <f>G59-X59-Y59</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60" spans="1:26">
       <c r="A60" s="17"/>
       <c r="B60" s="18"/>
-      <c r="C60" s="19"/>
+      <c r="C60" s="19" t="s">
+        <v>141</v>
+      </c>
       <c r="D60" s="19"/>
       <c r="E60" s="19"/>
-      <c r="F60" s="19"/>
-      <c r="G60" s="20"/>
-      <c r="H60" s="21"/>
-      <c r="I60" s="21"/>
+      <c r="F60" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="G60" s="8">
+        <v>4</v>
+      </c>
+      <c r="H60" s="21">
+        <v>3</v>
+      </c>
+      <c r="I60" s="21">
+        <v>1</v>
+      </c>
       <c r="J60" s="21"/>
       <c r="K60" s="21"/>
       <c r="L60" s="21"/>
@@ -3563,106 +3744,204 @@
       <c r="V60" s="21"/>
       <c r="W60" s="21"/>
       <c r="X60" s="11">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="Y60" s="20"/>
+        <f t="shared" si="2"/>
+        <v>4</v>
+      </c>
+      <c r="Y60" s="20">
+        <v>0</v>
+      </c>
       <c r="Z60" s="28">
         <f>G60-X60-Y60</f>
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="1:26" ht="12.6" thickBot="1">
-      <c r="A61" s="22"/>
-      <c r="B61" s="2" t="s">
-        <v>137</v>
-      </c>
-      <c r="C61" s="3"/>
-      <c r="D61" s="3"/>
-      <c r="E61" s="3"/>
-      <c r="F61" s="23">
-        <f t="shared" ref="F61:Z61" si="5">SUM(F2:F60)</f>
-        <v>0</v>
-      </c>
-      <c r="G61" s="23">
-        <f t="shared" si="5"/>
-        <v>322</v>
-      </c>
-      <c r="H61" s="23">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="I61" s="23">
-        <f t="shared" si="5"/>
-        <v>6</v>
-      </c>
-      <c r="J61" s="23">
-        <f t="shared" si="5"/>
+    <row r="61" spans="1:26">
+      <c r="A61" s="17"/>
+      <c r="B61" s="18"/>
+      <c r="C61" s="19" t="s">
+        <v>142</v>
+      </c>
+      <c r="D61" s="19"/>
+      <c r="E61" s="19"/>
+      <c r="F61" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="G61" s="8">
+        <v>16</v>
+      </c>
+      <c r="H61" s="21"/>
+      <c r="I61" s="21"/>
+      <c r="J61" s="21"/>
+      <c r="K61" s="21"/>
+      <c r="L61" s="21"/>
+      <c r="M61" s="21">
+        <v>1</v>
+      </c>
+      <c r="N61" s="21">
+        <v>1</v>
+      </c>
+      <c r="O61" s="21">
+        <v>1</v>
+      </c>
+      <c r="P61" s="21">
+        <v>1</v>
+      </c>
+      <c r="Q61" s="21">
+        <v>1</v>
+      </c>
+      <c r="R61" s="21">
+        <v>1</v>
+      </c>
+      <c r="S61" s="21">
+        <v>1</v>
+      </c>
+      <c r="T61" s="21">
+        <v>1</v>
+      </c>
+      <c r="U61" s="21">
+        <v>3</v>
+      </c>
+      <c r="V61" s="21">
+        <v>2</v>
+      </c>
+      <c r="W61" s="21"/>
+      <c r="X61" s="11">
+        <f t="shared" si="2"/>
+        <v>13</v>
+      </c>
+      <c r="Y61" s="20">
+        <v>0</v>
+      </c>
+      <c r="Z61" s="28">
+        <f>G61-X61-Y61</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="62" spans="1:26">
+      <c r="A62" s="17"/>
+      <c r="B62" s="18"/>
+      <c r="C62" s="19"/>
+      <c r="D62" s="19"/>
+      <c r="E62" s="19"/>
+      <c r="F62" s="19"/>
+      <c r="G62" s="20"/>
+      <c r="H62" s="21"/>
+      <c r="I62" s="21"/>
+      <c r="J62" s="21"/>
+      <c r="K62" s="21"/>
+      <c r="L62" s="21"/>
+      <c r="M62" s="21"/>
+      <c r="N62" s="21"/>
+      <c r="O62" s="21"/>
+      <c r="P62" s="21"/>
+      <c r="Q62" s="21"/>
+      <c r="R62" s="21"/>
+      <c r="S62" s="21"/>
+      <c r="T62" s="21"/>
+      <c r="U62" s="21"/>
+      <c r="V62" s="21"/>
+      <c r="W62" s="21"/>
+      <c r="X62" s="11">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="Y62" s="20"/>
+      <c r="Z62" s="28">
+        <f>G62-X62-Y62</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63" spans="1:26">
+      <c r="A63" s="22"/>
+      <c r="B63" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="C63" s="3"/>
+      <c r="D63" s="3"/>
+      <c r="E63" s="3"/>
+      <c r="F63" s="23">
+        <f t="shared" ref="F63:Z63" si="3">SUM(F2:F62)</f>
+        <v>0</v>
+      </c>
+      <c r="G63" s="23">
+        <f t="shared" si="3"/>
+        <v>357</v>
+      </c>
+      <c r="H63" s="23">
+        <f t="shared" si="3"/>
+        <v>3</v>
+      </c>
+      <c r="I63" s="23">
+        <f t="shared" si="3"/>
+        <v>7</v>
+      </c>
+      <c r="J63" s="23">
+        <f t="shared" si="3"/>
         <v>14</v>
       </c>
-      <c r="K61" s="23">
-        <f t="shared" si="5"/>
+      <c r="K63" s="23">
+        <f t="shared" si="3"/>
         <v>23</v>
       </c>
-      <c r="L61" s="23">
-        <f t="shared" si="5"/>
+      <c r="L63" s="23">
+        <f t="shared" si="3"/>
         <v>25</v>
       </c>
-      <c r="M61" s="23">
-        <f t="shared" si="5"/>
-        <v>38</v>
-      </c>
-      <c r="N61" s="23">
-        <f t="shared" si="5"/>
+      <c r="M63" s="23">
+        <f t="shared" si="3"/>
+        <v>45</v>
+      </c>
+      <c r="N63" s="23">
+        <f t="shared" si="3"/>
+        <v>32</v>
+      </c>
+      <c r="O63" s="23">
+        <f t="shared" si="3"/>
+        <v>27</v>
+      </c>
+      <c r="P63" s="23">
+        <f t="shared" si="3"/>
         <v>34</v>
       </c>
-      <c r="O61" s="23">
-        <f t="shared" si="5"/>
-        <v>16</v>
-      </c>
-      <c r="P61" s="23">
-        <f t="shared" si="5"/>
-        <v>2</v>
-      </c>
-      <c r="Q61" s="23">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="R61" s="23">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="S61" s="23">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="T61" s="23">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="U61" s="23">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="V61" s="23">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="W61" s="23">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="X61" s="23">
-        <f t="shared" si="5"/>
-        <v>111</v>
-      </c>
-      <c r="Y61" s="23">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="Z61" s="29">
-        <f t="shared" si="5"/>
-        <v>173</v>
+      <c r="Q63" s="23">
+        <f t="shared" si="3"/>
+        <v>15</v>
+      </c>
+      <c r="R63" s="23">
+        <f t="shared" si="3"/>
+        <v>7</v>
+      </c>
+      <c r="S63" s="23">
+        <f t="shared" si="3"/>
+        <v>12</v>
+      </c>
+      <c r="T63" s="23">
+        <f t="shared" si="3"/>
+        <v>34</v>
+      </c>
+      <c r="U63" s="23">
+        <f t="shared" si="3"/>
+        <v>34</v>
+      </c>
+      <c r="V63" s="23">
+        <f t="shared" si="3"/>
+        <v>47</v>
+      </c>
+      <c r="W63" s="23">
+        <f t="shared" si="3"/>
+        <v>5</v>
+      </c>
+      <c r="X63" s="23">
+        <f t="shared" si="3"/>
+        <v>361</v>
+      </c>
+      <c r="Y63" s="23">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="Z63" s="29">
+        <f t="shared" si="3"/>
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>